<commit_message>
Add employee codes for crew: Staff E001…, Workman W001…
The crew form now asks for a category (Staff or Workman) and fills in the
next free employee code for it: E001, E002 … for Staff, W001, W002 … for
Workmen (highest existing code + 1, so deleted codes are never reused).
The code stays editable.

- migration adds crew.emp_category / emp_code with a unique index on the code
- collision with a code another device just saved -> fetch next code, retry
- hand-typed duplicate code -> clear message in the form
- crew members can now be edited (✎), which is how existing crew get a code
- code shown in the Crew table and under names in Payroll; payroll search
  matches codes
- if the migration hasn't been run yet, saving explains what to run
- upload template gets Employee Category / Employee Code columns
- tests/test_crew_codes.py covers the above

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015GPF5QjF4KqBF14KeDDdnP
</commit_message>
<xml_diff>
--- a/SolarOps_Initial_Data_Upload_Template.xlsx
+++ b/SolarOps_Initial_Data_Upload_Template.xlsx
@@ -1,34 +1,51 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="Instructions" sheetId="1" r:id="rId2"/>
-    <sheet name="Customers" sheetId="2" r:id="rId3"/>
-    <sheet name="Crew" sheetId="3" r:id="rId4"/>
-    <sheet name="Inventory" sheetId="4" r:id="rId5"/>
-    <sheet name="Assignments" sheetId="5" r:id="rId6"/>
-    <sheet name="Payroll" sheetId="6" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crew" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payroll" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Instructions'!$A$1:$A$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customers'!$A$1:$O$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Crew'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Inventory'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Assignments'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Payroll'!$A$1:$I$3</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <name val="Calibri"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
       <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -50,20 +67,379 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetFormatPr defaultRowHeight="18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -74,49 +450,49 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Use one sheet per master data type. Replace the example rows, keep the header names, and save as .xlsx before uploading or copying into Supabase.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="0" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Required fields are marked with *. Dates use YYYY-MM-DD. Amounts and quantities should be numbers without currency symbols or commas.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="0" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Customers: payment status is Pending or Paid. Enter Amount Paid only when payment has been received.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="0" t="inlineStr">
-        <is>
-          <t>Crew: Employment Type is Permanent or Contract. Contract Amount is used only for contract workers.</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Crew: Employment Type is Permanent or Contract. Contract Amount is used only for contract workers. Employee Category is Staff or Workman; Employee Code is E001, E002 … for Staff and W001, W002 … for Workmen (leave blank to have the app number them).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="0" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Assignments: Work Done Status is Not Started, In Progress, or Completed.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="0" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Payroll: one row per crew member per month. Pay Period should be the first day of the month, such as 2026-06-01.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="0" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Delete the example rows before your final upload if they are not real records.</t>
         </is>
@@ -124,29 +500,34 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:A8"/>
-  <dataValidations count="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetFormatPr defaultRowHeight="18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="14" customWidth="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -227,73 +608,73 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>CUST-001</t>
         </is>
       </c>
-      <c r="B2" s="0" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Example Customer</t>
         </is>
       </c>
-      <c r="C2" s="0" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>+91 98765 43210</t>
         </is>
       </c>
-      <c r="D2" s="0" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>example@email.com</t>
         </is>
       </c>
-      <c r="E2" s="0" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="F2" s="0" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>3KW</t>
         </is>
       </c>
-      <c r="G2" s="0">
+      <c r="G2" t="n">
         <v>185000</v>
       </c>
-      <c r="H2" s="0" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="I2" s="0">
+      <c r="I2" t="n">
         <v>185000</v>
       </c>
-      <c r="J2" s="0" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="K2" s="0" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Payment Received</t>
         </is>
       </c>
-      <c r="L2" s="0" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>PMGSY-2026-0001</t>
         </is>
       </c>
-      <c r="M2" s="0" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>WO-2026-0001</t>
         </is>
       </c>
-      <c r="N2" s="0" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="O2" s="0" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Replace this example row</t>
         </is>
@@ -302,31 +683,37 @@
   </sheetData>
   <autoFilter ref="A1:O2"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="H2:H1000">
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Paid"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="N2:N1000">
+    <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetFormatPr defaultRowHeight="18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -337,152 +724,180 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Employee Category *</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Employee Code</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Name *</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Designation</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Monthly Salary</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Joining Date</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Employment Type</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Contract Amount</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Assigned Team</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>CREW-001</t>
         </is>
       </c>
-      <c r="B2" s="0" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>E001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Example Electrician</t>
         </is>
       </c>
-      <c r="C2" s="0" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Electrician</t>
         </is>
       </c>
-      <c r="D2" s="0" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>+91 90000 11001</t>
         </is>
       </c>
-      <c r="E2" s="0">
+      <c r="G2" t="n">
         <v>28000</v>
       </c>
-      <c r="F2" s="0" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="G2" s="0" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Permanent</t>
         </is>
       </c>
-      <c r="H2" s="0"/>
-      <c r="I2" s="0" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="J2" s="0" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K2" s="0" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Replace this example row</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="0" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>CREW-002</t>
         </is>
       </c>
-      <c r="B3" s="0" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Workman</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>W001</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>Example Installer</t>
         </is>
       </c>
-      <c r="C3" s="0" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Installer</t>
         </is>
       </c>
-      <c r="D3" s="0" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>+91 90000 11002</t>
         </is>
       </c>
-      <c r="E3" s="0"/>
-      <c r="F3" s="0" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="G3" s="0" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Contract</t>
         </is>
       </c>
-      <c r="H3" s="0">
+      <c r="J3" t="n">
         <v>3500</v>
       </c>
-      <c r="I3" s="0" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Team 2</t>
         </is>
       </c>
-      <c r="J3" s="0" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K3" s="0" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Contract Amount is per contract/job</t>
         </is>
@@ -490,30 +905,39 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K3"/>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="G2:G1000">
+  <dataValidations count="3">
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Permanent,Contract"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="J2:J1000">
+    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Staff,Workman"</formula1>
+    </dataValidation>
   </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetFormatPr defaultRowHeight="18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,41 +988,41 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>INV-001</t>
         </is>
       </c>
-      <c r="B2" s="0" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Example 450W Solar Panel</t>
         </is>
       </c>
-      <c r="C2" s="0" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Panel</t>
         </is>
       </c>
-      <c r="D2" s="0">
+      <c r="D2" t="n">
         <v>50</v>
       </c>
-      <c r="E2" s="0">
+      <c r="E2" t="n">
         <v>12500</v>
       </c>
-      <c r="F2" s="0">
+      <c r="F2" t="n">
         <v>10</v>
       </c>
-      <c r="G2" s="0" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Example Supplier</t>
         </is>
       </c>
-      <c r="H2" s="0" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>+91 90000 22001</t>
         </is>
       </c>
-      <c r="I2" s="0" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Replace this example row</t>
         </is>
@@ -606,25 +1030,30 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I2"/>
-  <dataValidations count="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetFormatPr defaultRowHeight="18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -685,57 +1114,57 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ASN-001</t>
         </is>
       </c>
-      <c r="B2" s="0" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>CUST-001</t>
         </is>
       </c>
-      <c r="C2" s="0" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Example Customer</t>
         </is>
       </c>
-      <c r="D2" s="0" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>PMGSY-2026-0001</t>
         </is>
       </c>
-      <c r="E2" s="0" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>WO-2026-0001</t>
         </is>
       </c>
-      <c r="F2" s="0" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G2" s="0" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="H2" s="0" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Assigned</t>
         </is>
       </c>
-      <c r="I2" s="0" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="J2" s="0" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="K2" s="0" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Replace this example row</t>
         </is>
@@ -744,29 +1173,35 @@
   </sheetData>
   <autoFilter ref="A1:K2"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="H2:H1000">
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Assigned,Unassigned,Rescheduled"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I2:I1000">
+    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Completed"</formula1>
     </dataValidation>
   </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetFormatPr defaultRowHeight="18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -817,86 +1252,85 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>PAY-2026-06-001</t>
         </is>
       </c>
-      <c r="B2" s="0" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>CREW-001</t>
         </is>
       </c>
-      <c r="C2" s="0" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Example Electrician</t>
         </is>
       </c>
-      <c r="D2" s="0" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="E2" s="0" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Monthly Salary</t>
         </is>
       </c>
-      <c r="F2" s="0">
+      <c r="F2" t="n">
         <v>28000</v>
       </c>
-      <c r="G2" s="0" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="H2" s="0" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="I2" s="0" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>June 2026 example</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="0" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>PAY-2026-07-001</t>
         </is>
       </c>
-      <c r="B3" s="0" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>CREW-001</t>
         </is>
       </c>
-      <c r="C3" s="0" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Example Electrician</t>
         </is>
       </c>
-      <c r="D3" s="0" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="E3" s="0" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Monthly Salary</t>
         </is>
       </c>
-      <c r="F3" s="0">
+      <c r="F3" t="n">
         <v>28000</v>
       </c>
-      <c r="G3" s="0" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="H3" s="0"/>
-      <c r="I3" s="0" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>July 2026 example</t>
         </is>
@@ -905,9 +1339,10 @@
   </sheetData>
   <autoFilter ref="A1:I3"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="G2:G1000">
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Paid"</formula1>
     </dataValidation>
   </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>